<commit_message>
feat: updating existing dairy livestock tests for shared code updates
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/5.2-organic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/5.2-organic-fertiliser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E913DBAC-EA2E-3441-9ABE-CA158C33DE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D485858-894E-9B48-9AC3-68495A050BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="760" windowWidth="50560" windowHeight="26020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2520" yWindow="1520" windowWidth="50560" windowHeight="26020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.2.1.1 (purchased_untraced)" sheetId="1" r:id="rId1"/>
@@ -15981,19 +15981,24 @@
         <v>1</v>
       </c>
       <c r="AR71">
+        <f>$BZ$64</f>
         <v>0.02</v>
       </c>
       <c r="AS71">
+        <f>X71+X72+X74</f>
         <v>0.48773949</v>
       </c>
       <c r="AT71">
+        <f>X73+X75</f>
         <v>5.241817E-2</v>
       </c>
       <c r="AU71">
-        <v>1.7061210600000001</v>
+        <f>Y71+Y72+Y74</f>
+        <v>1.6414287625030253</v>
       </c>
       <c r="AV71">
-        <v>0.22558537000000001</v>
+        <f>Y73+Y75</f>
+        <v>0.20102491308955134</v>
       </c>
       <c r="AW71" t="s">
         <v>228</v>
@@ -16052,11 +16057,11 @@
       </c>
       <c r="BQ71">
         <f>SUM(BN71:BN74)</f>
-        <v>24141.080124162781</v>
+        <v>23380.878795239161</v>
       </c>
       <c r="BR71">
         <f>SUM(BO71:BO74)</f>
-        <v>6035.2700310406935</v>
+        <v>5845.2196988097894</v>
       </c>
       <c r="BS71">
         <f>IF(ISBLANK(AJ71), "", IF(AJ71="wet", $BZ$67, $BZ$68))</f>
@@ -16068,11 +16073,11 @@
       </c>
       <c r="BU71">
         <f>IF(ISBLANK(A71), "", BQ71*BS71*BT71/1000)</f>
-        <v>0.22761589831353482</v>
+        <v>0.2204482857836835</v>
       </c>
       <c r="BV71">
         <f>IF(ISBLANK(AT71), "", BR71*BS71*BT71/1000)</f>
-        <v>5.6903974578383684E-2</v>
+        <v>5.5112071445920875E-2</v>
       </c>
     </row>
     <row r="72" spans="1:78" x14ac:dyDescent="0.2">
@@ -16168,18 +16173,18 @@
       </c>
       <c r="BL72">
         <f>((AA71 * AU71 * 365) + (AC71 * AV71 * 281)  + (AC71 *AF71 * 84)) *BH72</f>
-        <v>9950.9205764920025</v>
+        <v>9548.6368372672259</v>
       </c>
       <c r="BM72">
         <v>0</v>
       </c>
       <c r="BN72">
         <f>((BK72 + BL72) * (1 - BI72 -BJ72)- BM72) *AH$11</f>
-        <v>9504.5921746779386</v>
+        <v>9205.2930726947034</v>
       </c>
       <c r="BO72">
         <f>((BK72 + BL72) * (1 - BI72 -BJ72)- BM72) *(1 - AH$11)</f>
-        <v>2376.1480436694837</v>
+        <v>2301.3232681736754</v>
       </c>
     </row>
     <row r="73" spans="1:78" x14ac:dyDescent="0.2">
@@ -16283,18 +16288,18 @@
       </c>
       <c r="BL73">
         <f>((AA71 * AU71 * 365) + (AC71 * AV71 * 281)  + (AC71 *AF71 * 84)) *BH73</f>
-        <v>14215.600823560002</v>
+        <v>13640.909767524608</v>
       </c>
       <c r="BM73">
         <v>0</v>
       </c>
       <c r="BN73">
         <f>((BK73 + BL73) * (1 - BI73 -BJ73)- BM73) *AH$11</f>
-        <v>11679.990383628803</v>
+        <v>11312.188107766153</v>
       </c>
       <c r="BO73">
         <f>((BK73 + BL73) * (1 - BI73 -BJ73)- BM73) *(1 - AH$11)</f>
-        <v>2919.9975959071999</v>
+        <v>2828.0470269415373</v>
       </c>
     </row>
     <row r="74" spans="1:78" x14ac:dyDescent="0.2">
@@ -16387,19 +16392,19 @@
       </c>
       <c r="BL74">
         <f>((AA71 * AU71 * 365) + (AC71 * AV71 * 281)  + (AC71 *AF71 * 84)) *BH74</f>
-        <v>4264.6802470680004</v>
+        <v>4092.2729302573821</v>
       </c>
       <c r="BM74">
         <f>(BL74+ BK74) *AQ71 *AR71</f>
-        <v>109.49990984652001</v>
+        <v>106.05176351030765</v>
       </c>
       <c r="BN74">
         <f>((BK74 + BL74) * (1 - BI74 -BJ74)- BM74) *AH$11</f>
-        <v>2956.4975658560406</v>
+        <v>2863.3976147783069</v>
       </c>
       <c r="BO74">
         <f>((BK74 + BL74) * (1 - BI74 -BJ74)- BM74) *(1 - AH$11)</f>
-        <v>739.12439146400993</v>
+        <v>715.84940369457649</v>
       </c>
     </row>
     <row r="75" spans="1:78" x14ac:dyDescent="0.2">
@@ -16500,7 +16505,7 @@
       </c>
       <c r="BL75">
         <f>((AA71 * AU71 * 365) + (AC71 * AV71 * 281)  + (AC71 *AF71 * 84)) *BH75</f>
-        <v>28431.201647120004</v>
+        <v>27281.819535049217</v>
       </c>
       <c r="BM75">
         <v>0</v>
@@ -17844,7 +17849,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="C3:CH10 C16:E19 C12:E12 BW12:CH12 A3:A96 C77:CH85 C51:E54 C11:E11 G11:I11 G12:I12 C13:E13 G13:I13 C14:E14 G14:I14 C15:E15 G15:I15 G16:I18 C20:E20 G20:I20 C21:E25 G21:I25 C26:E30 G26:I30 C31:E35 G31:I35 C36:E40 G36:I38 C41:E45 G41:I45 C46:E50 G46:I50 C55:E55 G55:I55 G53:I54 C56:E60 G56:CH58 C61:E65 G61:I65 C66:E70 G66:I70 C71:E75 G73:I75 C91:CH91 C86:E90 G86:CH90 C92:E96 G92:CH96 G19:I19 CA19:CH19 CA20:CD20 CA21:CD25 G51:I51 BW51:CD51 G52:I52 BO52:CD52 BM52 AV51:BU51 Z51:AT51 R51:X51 L51:P51 G71:I71 BV71:CH71 BR71:BT71 G72:I72 BO72:CH72 BM72 K11:CH11 G39:I40 CA39:CD40 CA41:CD45 K12:BM12 K13:CH13 K14:CH14 K15:CH15 K16:CH18 K20:BW20 K19:BW19 K21:BW25 K26:CD30 K31:CD35 K36:CD38 K39:BW40 K41:BW45 K46:CD50 K55:CH55 K53:CD54 K52:BK52 K61:CH65 K66:L70 K73:L75 K71:L71 K72:L72 O66:O70 O71 C76:L76 N76:CH76 O73:O75 O72 Q66:CH70 R71 R73:R75 R72 G60:CH60 G59:R59 T59:CH59 X71 X73:X75 X72 AA71:BP71 AA73:CH75 AA72:BK72 BO12:BU12" numberStoredAsText="1"/>
+    <ignoredError sqref="C3:CH10 C16:E19 C12:E12 BW12:CH12 A3:A96 C77:CH85 C51:E54 C11:E11 G11:I11 G12:I12 C13:E13 G13:I13 C14:E14 G14:I14 C15:E15 G15:I15 G16:I18 C20:E20 G20:I20 C21:E25 G21:I25 C26:E30 G26:I30 C31:E35 G31:I35 C36:E40 G36:I38 C41:E45 G41:I45 C46:E50 G46:I50 C55:E55 G55:I55 G53:I54 C56:E60 G56:CH58 C61:E65 G61:I65 C66:E70 G66:I70 C71:E75 G73:I75 C91:CH91 C86:E90 G86:CH90 C92:E96 G92:CH96 G19:I19 CA19:CH19 CA20:CD20 CA21:CD25 G51:I51 BW51:CD51 G52:I52 BO52:CD52 BM52 AV51:BU51 Z51:AT51 R51:X51 L51:P51 G71:I71 BV71:CH71 BR71:BT71 G72:I72 BO72:CH72 BM72 K11:CH11 G39:I40 CA39:CD40 CA41:CD45 K12:BM12 K13:CH13 K14:CH14 K15:CH15 K16:CH18 K20:BW20 K19:BW19 K21:BW25 K26:CD30 K31:CD35 K36:CD38 K39:BW40 K41:BW45 K46:CD50 K55:CH55 K53:CD54 K52:BK52 K61:CH65 K66:L70 K73:L75 K71:L71 K72:L72 O66:O70 O71 C76:L76 N76:CH76 O73:O75 O72 Q67:CH70 R71 R73:R75 R72 G60:CH60 G59:R59 T59:CH59 X71 X73:X75 X72 AA71:AQ71 AA73:CH75 AA72:BK72 BO12:BU12 Q66:AT66 AV66:CH66 AW71:BP71" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(calculators): reverted to initial allocation schema, plus constant cleanup
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/5.2-organic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/5.2-organic-fertiliser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/5.2-organic-fertiliser-n2o/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D485858-894E-9B48-9AC3-68495A050BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159333E7-5453-5A4F-BBE6-2AA0B367FF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="1520" windowWidth="50560" windowHeight="26020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15900" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.2.1.1 (purchased_untraced)" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="5.2.1.1 (poultry)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -60,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="483">
   <si>
     <t>Table A.2.1.4</t>
   </si>
@@ -1506,6 +1505,9 @@
   </si>
   <si>
     <t>0.3003 </t>
+  </si>
+  <si>
+    <t>Pasture range and paddock (free range)</t>
   </si>
 </sst>
 </file>
@@ -18399,7 +18401,7 @@
       </c>
       <c r="AD11">
         <f>AA13*(1 - V13 - U13)</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AE11">
         <f>AA14*(1 - V14 - U14)</f>
@@ -18445,7 +18447,7 @@
       </c>
       <c r="AR11">
         <f>SUM(AP11:AP15)</f>
-        <v>266.00820711536636</v>
+        <v>266.68247516336635</v>
       </c>
       <c r="AS11">
         <f>SUM(AQ11:AQ14)</f>
@@ -18461,7 +18463,7 @@
       </c>
       <c r="AV11">
         <f>IF(ISBLANK(D11), "", AR11*AT11*AU11/1000)</f>
-        <v>2.5080773813734541E-3</v>
+        <v>2.5144347658260257E-3</v>
       </c>
       <c r="AW11">
         <f>IF(ISBLANK(D11), "", AS11*AT11*AU11/1000)</f>
@@ -18548,7 +18550,7 @@
         <v>0</v>
       </c>
       <c r="AA12">
-        <f t="shared" ref="AA12:AA14" si="4">SUM(W12:Z12)</f>
+        <f>SUM(W12:Z12)</f>
         <v>422.67684800000001</v>
       </c>
       <c r="AF12" s="5" t="s">
@@ -18645,7 +18647,7 @@
       </c>
       <c r="U13">
         <f>VLOOKUP(S13, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V13">
         <f>VLOOKUP(S13, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -18668,7 +18670,7 @@
         <v>0</v>
       </c>
       <c r="AA13">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="AA12:AA14" si="4">SUM(W13:Z13)</f>
         <v>35.487791999999999</v>
       </c>
       <c r="AF13" s="5" t="s">
@@ -18791,7 +18793,7 @@
       </c>
       <c r="AD14">
         <f>SUM(AB11:AD11)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AF14" t="s">
         <v>425</v>
@@ -18841,14 +18843,14 @@
       </c>
       <c r="AJ15">
         <f>AG15*AB11+AH15*AC11+AI15*AD11</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AO15">
         <v>0</v>
       </c>
       <c r="AP15">
         <f>AJ15</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="BD15" s="4" t="s">
         <v>372</v>
@@ -18872,7 +18874,7 @@
       </c>
       <c r="AJ16">
         <f>SUM(AJ11:AJ15)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AY16" t="s">
         <v>3</v>
@@ -19000,7 +19002,7 @@
       </c>
       <c r="AD21">
         <f>AA23*(1 - V23 - U23)</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AE21">
         <f>AA24*(1 - V24 - U24)</f>
@@ -19046,7 +19048,7 @@
       </c>
       <c r="AR21">
         <f>SUM(AP21:AP25)</f>
-        <v>266.08123795537915</v>
+        <v>266.7555060033792</v>
       </c>
       <c r="AS21">
         <f>SUM(AQ21:AQ24)</f>
@@ -19062,7 +19064,7 @@
       </c>
       <c r="AV21">
         <f>IF(ISBLANK(D21), "", AR21*AT21*AU21/1000)</f>
-        <v>2.5087659578650031E-3</v>
+        <v>2.5151233423175751E-3</v>
       </c>
       <c r="AW21">
         <f>IF(ISBLANK(D21), "", AS21*AT21*AU21/1000)</f>
@@ -19233,7 +19235,7 @@
       </c>
       <c r="U23">
         <f>VLOOKUP(S23, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V23">
         <f>VLOOKUP(S23, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -19376,7 +19378,7 @@
       </c>
       <c r="AD24">
         <f>SUM(AB21:AD21)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AF24" t="s">
         <v>425</v>
@@ -19432,14 +19434,14 @@
       </c>
       <c r="AJ25">
         <f>AG25*AB21+AH25*AC21+AI25*AD21</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AO25">
         <v>0</v>
       </c>
       <c r="AP25">
         <f>AJ25</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AY25" s="5" t="s">
         <v>406</v>
@@ -19467,7 +19469,7 @@
       </c>
       <c r="AJ26">
         <f>SUM(AJ21:AJ25)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AY26" s="5" t="s">
         <v>407</v>
@@ -19630,7 +19632,7 @@
       </c>
       <c r="AD31">
         <f>AA33*(1 - V33 - U33)</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AE31">
         <f>AA34*(1 - V34 - U34)</f>
@@ -19676,7 +19678,7 @@
       </c>
       <c r="AR31">
         <f>SUM(AP31:AP35)</f>
-        <v>266.00820711536636</v>
+        <v>266.68247516336635</v>
       </c>
       <c r="AS31">
         <f>SUM(AQ31:AQ34)</f>
@@ -19692,7 +19694,7 @@
       </c>
       <c r="AV31">
         <f>IF(ISBLANK(D31), "", AR31*AT31*AU31/1000)</f>
-        <v>2.0900644844778784E-3</v>
+        <v>2.0953623048550214E-3</v>
       </c>
       <c r="AW31">
         <f>IF(ISBLANK(D31), "", AS31*AT31*AU31/1000)</f>
@@ -19873,7 +19875,7 @@
       </c>
       <c r="U33">
         <f>VLOOKUP(S33, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V33">
         <f>VLOOKUP(S33, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -20012,7 +20014,7 @@
       </c>
       <c r="AD34">
         <f>SUM(AB31:AD31)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AF34" t="s">
         <v>425</v>
@@ -20050,7 +20052,7 @@
         <v>0.4</v>
       </c>
       <c r="BA34" s="5">
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="35" spans="1:53" x14ac:dyDescent="0.2">
@@ -20062,14 +20064,14 @@
       </c>
       <c r="AJ35">
         <f>AG35*AB31+AH35*AC31+AI35*AD31</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AO35">
         <v>0</v>
       </c>
       <c r="AP35">
         <f>AJ35</f>
-        <v>20.582919359999998</v>
+        <v>21.257187408</v>
       </c>
       <c r="AY35" s="5" t="s">
         <v>426</v>
@@ -20099,7 +20101,7 @@
       </c>
       <c r="AJ36">
         <f>SUM(AJ31:AJ35)</f>
-        <v>431.84642033599999</v>
+        <v>432.52068838399998</v>
       </c>
       <c r="AY36" s="5" t="s">
         <v>427</v>
@@ -20131,6 +20133,14 @@
       </c>
       <c r="BA38" s="5">
         <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="AY39" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="BA39" s="5">
+        <v>0.02</v>
       </c>
     </row>
     <row r="41" spans="1:53" x14ac:dyDescent="0.2">
@@ -20461,7 +20471,7 @@
       </c>
       <c r="U43">
         <f>VLOOKUP(S43, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V43">
         <f>VLOOKUP(S43, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -20760,7 +20770,7 @@
       </c>
       <c r="AD51">
         <f>AA53*(1 - V53 - U53)</f>
-        <v>94.684118399999988</v>
+        <v>97.785839519999996</v>
       </c>
       <c r="AE51">
         <f>AA54*(1 - V54 - U54)</f>
@@ -20806,7 +20816,7 @@
       </c>
       <c r="AR51">
         <f>SUM(AP51:AP55)</f>
-        <v>378.45926564966396</v>
+        <v>381.56098676966394</v>
       </c>
       <c r="AS51">
         <f>SUM(AQ51:AQ54)</f>
@@ -20822,7 +20832,7 @@
       </c>
       <c r="AV51">
         <f>IF(ISBLANK(D51), "", AR51*AT51*AU51/1000)</f>
-        <v>3.5683302189825463E-3</v>
+        <v>3.5975750181139743E-3</v>
       </c>
       <c r="AW51">
         <f>IF(ISBLANK(D51), "", AS51*AT51*AU51/1000)</f>
@@ -20985,7 +20995,7 @@
       </c>
       <c r="U53">
         <f>VLOOKUP(S53, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V53">
         <f>VLOOKUP(S53, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -21115,7 +21125,7 @@
       </c>
       <c r="AD54">
         <f>SUM(AB51:AD51)</f>
-        <v>589.85624431999997</v>
+        <v>592.95796543999995</v>
       </c>
       <c r="AF54" t="s">
         <v>425</v>
@@ -21156,14 +21166,14 @@
       </c>
       <c r="AJ55">
         <f>AG55*AB51+AH55*AC51+AI55*AD51</f>
-        <v>94.684118399999988</v>
+        <v>97.785839519999996</v>
       </c>
       <c r="AO55">
         <v>0</v>
       </c>
       <c r="AP55">
         <f>AJ55</f>
-        <v>94.684118399999988</v>
+        <v>97.785839519999996</v>
       </c>
     </row>
     <row r="56" spans="1:49" x14ac:dyDescent="0.2">
@@ -21184,7 +21194,7 @@
       </c>
       <c r="AJ56">
         <f>SUM(AJ51:AJ55)</f>
-        <v>589.85624431999997</v>
+        <v>592.95796543999995</v>
       </c>
     </row>
     <row r="61" spans="1:49" x14ac:dyDescent="0.2">
@@ -21279,7 +21289,7 @@
       </c>
       <c r="AD61">
         <f>AA63*(1 - V63 - U63)</f>
-        <v>14.732927999999998</v>
+        <v>15.215558399999999</v>
       </c>
       <c r="AE61">
         <f>AA64*(1 - V64 - U64)</f>
@@ -21325,7 +21335,7 @@
       </c>
       <c r="AR61">
         <f>SUM(AP61:AP65)</f>
-        <v>190.81681904640001</v>
+        <v>191.29944944640002</v>
       </c>
       <c r="AS61">
         <f>SUM(AQ61:AQ64)</f>
@@ -21341,7 +21351,7 @@
       </c>
       <c r="AV61">
         <f>IF(ISBLANK(D61), "", AR61*AT61*AU61/1000)</f>
-        <v>1.7991300081517717E-3</v>
+        <v>1.8036805233517716E-3</v>
       </c>
       <c r="AW61">
         <f>IF(ISBLANK(D61), "", AS61*AT61*AU61/1000)</f>
@@ -21500,7 +21510,7 @@
       </c>
       <c r="U63">
         <f>VLOOKUP(S63, $AY$32:$BA$38, 3, FALSE)</f>
-        <v>0.02</v>
+        <v>1E-3</v>
       </c>
       <c r="V63">
         <f>VLOOKUP(S63, $AY$32:$AZ$38, 2, FALSE)</f>
@@ -21628,7 +21638,7 @@
       </c>
       <c r="AD64">
         <f>SUM(AB61:AD61)</f>
-        <v>310.00876160000007</v>
+        <v>310.49139200000008</v>
       </c>
       <c r="AF64" t="s">
         <v>425</v>
@@ -21669,14 +21679,14 @@
       </c>
       <c r="AJ65">
         <f>AG65*AB61+AH65*AC61+AI65*AD61</f>
-        <v>14.732927999999998</v>
+        <v>15.215558399999999</v>
       </c>
       <c r="AO65">
         <v>0</v>
       </c>
       <c r="AP65">
         <f>AJ65</f>
-        <v>14.732927999999998</v>
+        <v>15.215558399999999</v>
       </c>
     </row>
     <row r="66" spans="32:42" x14ac:dyDescent="0.2">
@@ -21697,7 +21707,7 @@
       </c>
       <c r="AJ66">
         <f>SUM(AJ61:AJ65)</f>
-        <v>310.00876160000007</v>
+        <v>310.49139200000008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>